<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-07 Le croissant de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-07.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-07.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La gaufre de la place de Mila</t>
+          <t>Le croissant de Mila</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>place du village, fer à gaufres</t>
+          <t>rue tiède, farine sur la vitre, rayon blanc, boulangerie, comptoir de marbre, croissant</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut la gaufre dorée qui sort du fer. Elle dit bonjour, s'il te plaît, merci. La vanille reste sur ses doigts.</t>
+          <t>Un rayon blanc tient sur la vitre. La farine y reste. Sur la pointe, un éclat de croissant brille. Mila veut le croissant maintenant. Elle parle trop vite, sans le mot : la dame n'a pas levé les yeux. Elle refuse de foncer, dit bonjour. Merci vécu. Le sac glisse. Un éclat de croissant reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un pigeon picore une miette sur la place. Le fer à gaufres souffle un peu de vapeur. Ça sent la vanille, tout chaud. Un banc de pierre est froid au soleil. Papa tient la main de Mila. Sa main est un peu collante, déjà. Tu as senti la vanille, Mila ? Ça sent le gâteau. C'est le fer. La vapeur fait un petit nuage. Il part vers les pigeons. Tu vois le nuage, Mila ? Il s'en va. En ce moment, Mila s'arrête près du fer. Une gaufre dorée est encore fermée. Le fer est chaud, tout silencieux. Je la veux, papa. On reste près du fer. On attend un peu. La dame tourne le fer. Le bois de la poignée est lisse. Mila se tient près de maman. Le fer s'ouvre. La gaufre est dorée, avec des trous. Un peu de vapeur monte encore. Elle a des trous. Comme le fer. Tu demandes, Mila.</t>
+          <t>Un rayon blanc tient sur la vitre. La farine y reste, sans tomber. Sous les chaussures, la rue est tiède. Ça sent le beurre, papa. Tu le sens, toi ? Oui, chaud. Le soleil touche tes joues. Elles sont tièdes, maman. Papa tient la main de Mila. Sa paume a un peu de farine. Tu as vu la farine, Mila ? Elle ne tombe pas, papa. Non. Elle reste sur la vitre. Derrière le verre, les croissants dorés attendent. Un croissant a une pointe plus brune. Celui-là, papa. Sur la pointe, un éclat de croissant brille. Il brille, maman ! Tu le vois, sur le croissant ? Oui, près de la pointe. Je le veux, maintenant. En ce moment, Mila pousse la porte. Une cloche fait ding. La chaleur entre dans les manches. Il est chaud ici. On reste près du marbre ? Oui. La dame essuie le comptoir de marbre. Le marbre est froid, malgré le four. Elle a un torchon gris à la main. Celui-là ! Mila parle trop vite vers le marbre. Sa voix se mélange au torchon. La dame n'a pas levé les yeux. Oh. Le croissant reste derrière le verre. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le croissant est derrière le verre. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un pigeon picore une miette sur la place. Le fer à gaufres souffle un peu de vapeur. Ça sent la vanille, tout chaud. Un banc de pierre est froid au soleil. Papa tient la main de Mila. Sa main est un peu collante, déjà. Tu as senti la vanille, Mila ? Ça sent le gâteau. C'est le fer. La vapeur fait un petit nuage. Il part vers les pigeons. Tu vois le nuage, Mila ? Il s'en va. En ce moment, Mila s'arrête près du fer. Une gaufre dorée est encore fermée. Le fer est chaud, tout silencieux. Je la veux, papa. On reste près du fer. On attend un peu. La dame tourne le fer. Le bois de la poignée est lisse. Mila se tient près de maman. Le fer s'ouvre. La gaufre est dorée, avec des trous. Un peu de vapeur monte encore. Elle a des trous. Comme le fer. Tu demandes, Mila.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon blanc tient sur la vitre. La farine y reste, sans tomber. Sous les chaussures, la rue est tiède. Ça sent le beurre, papa. Tu le sens, toi ? Oui, chaud. Le soleil touche tes joues. Elles sont tièdes, maman. Papa tient la main de Mila. Sa paume a un peu de farine. Tu as vu la farine, Mila ? Elle ne tombe pas, papa. Non. Elle reste sur la vitre. Derrière le verre, les croissants dorés attendent. Un croissant a une pointe plus brune. Celui-là, papa. Sur la pointe, un &lt;emphasis level="moderate"&gt;éclat de croissant&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur le croissant ? Oui, près de la pointe. Je le veux, maintenant. En ce moment, Mila pousse la porte. Une cloche fait ding. La chaleur entre dans les manches. Il est chaud ici. On reste près du marbre ? Oui. La dame essuie le comptoir de marbre. Le marbre est froid, malgré le four. Elle a un torchon gris à la main. Celui-là ! Mila parle trop vite vers le marbre. Sa voix se mélange au torchon. La dame n'a pas levé les yeux. Oh. Le croissant reste derrière le verre. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le croissant est derrière le verre. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fanny entre à la boulangerie. Papa tient sa main. Fanny dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. L'odeur du pain est chaude. Fanny pointe un croissant. Elle dit : s'il te plaît. La dame tend le sac. Fanny dit : merci. Papa sourit. Ils sortent. Le croissant est tiède. Fanny répète : bonjour. S'il te plaît. Merci. Maman les attend. Fanny dit : merci, maman. Maman dit : bonjour, Fanny. Ils rentrent.&lt;/slow&gt; [pause]</t>
+          <t>Un rayon blanc tient sur la vitre. La farine y reste, sans tomber. Sous les chaussures, la rue est tiède. Ça sent le beurre, papa. Tu le sens, toi ? Oui, chaud. Le soleil touche tes joues. Elles sont tièdes, maman. Papa tient la main de Mila. Sa paume a un peu de farine. Tu as vu la farine, Mila ? Elle ne tombe pas, papa. Non. Elle reste sur la vitre. Derrière le verre, les croissants dorés attendent. Un croissant a une pointe plus brune. Celui-là, papa. Sur la pointe, un &lt;emphasis&gt;éclat de croissant&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur le croissant ? Oui, près de la pointe. Je le veux, maintenant. En ce moment, Mila pousse la porte. Une cloche fait ding. La chaleur entre dans les manches. Il est chaud ici. On reste près du marbre ? Oui. La dame essuie le comptoir de marbre. Le marbre est froid, malgré le four. Elle a un torchon gris à la main. Celui-là ! Mila parle trop vite vers le marbre. Sa voix se mélange au torchon. La dame n'a pas levé les yeux. Oh. Le croissant reste derrière le verre. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le croissant est derrière le verre. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de croissant</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,44 +1324,65 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_croissant_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un pigeon picore une miette sur la place.
-narrateur|Le fer à gaufres souffle un peu de vapeur.
-narrateur|Ça sent la vanille, tout chaud.
-narrateur|Un banc de pierre est froid au soleil.
+          <t>narrateur|Un rayon blanc tient sur la vitre.
+narrateur|La farine y reste, sans tomber.
+narrateur|Sous les chaussures, la rue est tiède.
+enfant-f|Ça sent le beurre, papa.
+papa|Tu le sens, toi ?
+enfant-f|Oui, chaud.
+maman|Le soleil touche tes joues.
+enfant-f|Elles sont tièdes, maman.
 narrateur|Papa tient la main de Mila.
-narrateur|Sa main est un peu collante, déjà.
-maman|Tu as senti la vanille, Mila ?
-enfant-f|Ça sent le gâteau.
-papa|C'est le fer.
-narrateur|La vapeur fait un petit nuage.
-narrateur|Il part vers les pigeons.
-papa|Tu vois le nuage, Mila ?
-enfant-f|Il s'en va.
-narrateur|En ce moment, Mila s'arrête près du fer.
-narrateur|Une gaufre dorée est encore fermée.
-narrateur|Le fer est chaud, tout silencieux.
-enfant-f|Je la veux, papa.
-papa|On reste près du fer.
-maman|On attend un peu.
-narrateur|La dame tourne le fer.
-narrateur|Le bois de la poignée est lisse.
-narrateur|Mila se tient près de maman.
-narrateur|Le fer s'ouvre.
-narrateur|La gaufre est dorée, avec des trous.
-narrateur|Un peu de vapeur monte encore.
-enfant-f|Elle a des trous.
-papa|Comme le fer.
-maman|Tu demandes, Mila.</t>
+narrateur|Sa paume a un peu de farine.
+papa|Tu as vu la farine, Mila ?
+enfant-f|Elle ne tombe pas, papa.
+papa|Non.
+papa|Elle reste sur la vitre.
+narrateur|Derrière le verre, les croissants dorés attendent.
+narrateur|Un croissant a une pointe plus brune.
+enfant-f|Celui-là, papa.
+narrateur|Sur la pointe, un éclat de croissant brille.
+enfant-f|Il brille, maman !
+maman|Tu le vois, sur le croissant ?
+enfant-f|Oui, près de la pointe.
+enfant-f|Je le veux, maintenant.
+narrateur|En ce moment, Mila pousse la porte.
+narrateur|Une cloche fait ding.
+narrateur|La chaleur entre dans les manches.
+enfant-f|Il est chaud ici.
+papa|On reste près du marbre ?
+enfant-f|Oui.
+narrateur|La dame essuie le comptoir de marbre.
+narrateur|Le marbre est froid, malgré le four.
+narrateur|Elle a un torchon gris à la main.
+enfant-f|Celui-là !
+narrateur|Mila parle trop vite vers le marbre.
+narrateur|Sa voix se mélange au torchon.
+narrateur|La dame n'a pas levé les yeux.
+enfant-f|Oh.
+narrateur|Le croissant reste derrière le verre.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je le prends !
+maman|Le croissant est derrière le verre.
+papa|Tu le vois, Mila ?
+narrateur|Les épaules de Mila tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>vapeur,place</t>
+          <t>cloche,pas</t>
         </is>
       </c>
     </row>
@@ -1388,17 +1409,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Mila veut la gaufre. Que dit-elle ?</t>
+          <t>Mila parle à la dame. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila veut la gaufre. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fanny parle à la dame. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1423,7 +1444,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle dit bonjour. Que dit Mila ?</t>
+          <t>Bonjour, s'il te plaît, merci. Que dit Mila ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1461,7 +1482,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1469,10 +1490,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1487,34 +1508,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1523,13 +1548,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1539,12 +1564,12 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_dit_bonjour_a_la_dame; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Mila veut la gaufre.
+          <t>narrateur|Mila parle à la dame.
 narrateur|Que dit-elle ?</t>
         </is>
       </c>
@@ -1572,17 +1597,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une gaufre, s'il te plaît. Celle qui est dorée. La dame glisse la gaufre dans un papier. Le papier est chaud, un peu gras. Merci. Merci. Mila tient le papier contre son manteau. Ça sent la vanille, tout près. Elle est chaude, papa. Oui. La vapeur est sur ton nez. Ça chatouille. Un tout petit nuage. Le pigeon n'est plus sur la miette. Le banc de pierre reste froid. On s'assoit un moment ? Oui, maman. Le papier craque sur les genoux. Tu le tiens des deux mains. Oui, papa. Une miette de vanille reste sur le papier.</t>
+          <t>Mila avance trop vite vers le marbre. Celui-là, maintenant ! Sa voix se mélange au torchon. Oh. Le croissant reste derrière le verre. La dame essuie, sans lever les yeux. Mila refuse de foncer. Elle referme la main. Elle écoute la cloche, un instant. Tu veux venir près du marbre ? Papa s'accroupit à la même hauteur. Mila pose un pied sur le pas. Le marbre est froid sous l'air chaud. Bonjour. Celui-là. S'il te plaît. La dame pose le torchon. Elle lève les yeux. Une main glisse le croissant dans un sac. Le sac est chaud, un peu gras. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le four. Le croissant est à moi. Il est dans tes mains. Mila pose une main sur le sac. Le papier est un peu rêche. Sur le sac, un éclat de croissant tient. La cloche se tait.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une gaufre, s'il te plaît. Celle qui est dorée. La dame glisse la gaufre dans un papier. Le papier est chaud, un peu gras. Merci. Merci. Mila tient le papier contre son manteau. Ça sent la vanille, tout près. Elle est chaude, papa. Oui. La vapeur est sur ton nez. Ça chatouille. Un tout petit nuage. Le pigeon n'est plus sur la miette. Le banc de pierre reste froid. On s'assoit un moment ? Oui, maman. Le papier craque sur les genoux. Tu le tiens des deux mains. Oui, papa. Une miette de vanille reste sur le papier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila avance trop vite vers le marbre. Celui-là, maintenant ! Sa voix se mélange au torchon. Oh. Le croissant reste derrière le verre. La dame essuie, sans lever les yeux. Mila refuse de foncer. Elle referme la main. Elle écoute la cloche, un instant. Tu veux venir près du marbre ? Papa s'accroupit à la même hauteur. Mila pose un pied sur le pas. Le marbre est froid sous l'air chaud. &lt;emphasis level="moderate"&gt;Bonjour&lt;/emphasis&gt;. Celui-là. S'il te plaît. La dame pose le torchon. Elle lève les yeux. Une main glisse le croissant dans un sac. Le sac est chaud, un peu gras. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le four. Le croissant est à moi. Il est dans tes mains. Mila pose une main sur le sac. Le papier est un peu rêche. Sur le sac, un éclat de croissant tient. La cloche se tait.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fanny a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Elle a dit s'il te plaît. Elle a dit merci. Papa et maman ont entendu.&lt;/slow&gt; [pause]</t>
+          <t>Mila avance trop vite vers le marbre. Celui-là, maintenant ! Sa voix se mélange au torchon. Oh. Le croissant reste derrière le verre. La dame essuie, sans lever les yeux. Mila refuse de foncer. Elle referme la main. Elle écoute la cloche, un instant. Tu veux venir près du marbre ? Papa s'accroupit à la même hauteur. Mila pose un pied sur le pas. Le marbre est froid sous l'air chaud. &lt;emphasis&gt;Bonjour&lt;/emphasis&gt;. Celui-là. S'il te plaît. La dame pose le torchon. Elle lève les yeux. Une main glisse le croissant dans un sac. Le sac est chaud, un peu gras. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Ça sent le beurre et le four. Le croissant est à moi. Il est dans tes mains. Mila pose une main sur le sac. Le papier est un peu rêche. Sur le sac, un éclat de croissant tient. La cloche se tait. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1629,18 +1654,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1663,30 +1688,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>Bonjour</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1695,10 +1720,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1707,43 +1732,53 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=bonjour_ouvre_le_sac; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Bonjour.
-papa|Bonjour.
-enfant-f|Une gaufre, s'il te plaît.
-enfant-f|Celle qui est dorée.
-narrateur|La dame glisse la gaufre dans un papier.
-narrateur|Le papier est chaud, un peu gras.
-enfant-f|Merci.
-maman|Merci.
-narrateur|Mila tient le papier contre son manteau.
-narrateur|Ça sent la vanille, tout près.
-enfant-f|Elle est chaude, papa.
-papa|Oui.
-maman|La vapeur est sur ton nez.
-enfant-f|Ça chatouille.
-papa|Un tout petit nuage.
-narrateur|Le pigeon n'est plus sur la miette.
-narrateur|Le banc de pierre reste froid.
-maman|On s'assoit un moment ?
-enfant-f|Oui, maman.
-narrateur|Le papier craque sur les genoux.
-papa|Tu le tiens des deux mains.
-enfant-f|Oui, papa.
-narrateur|Une miette de vanille reste sur le papier.</t>
+          <t>narrateur|Mila avance trop vite vers le marbre.
+enfant-f|Celui-là, maintenant !
+narrateur|Sa voix se mélange au torchon.
+enfant-f|Oh.
+narrateur|Le croissant reste derrière le verre.
+narrateur|La dame essuie, sans lever les yeux.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la main.
+narrateur|Elle écoute la cloche, un instant.
+papa|Tu veux venir près du marbre ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Mila pose un pied sur le pas.
+narrateur|Le marbre est froid sous l'air chaud.
+enfant-f|Bonjour.
+enfant-f|Celui-là.
+enfant-f|S'il te plaît.
+narrateur|La dame pose le torchon.
+narrateur|Elle lève les yeux.
+narrateur|Une main glisse le croissant dans un sac.
+narrateur|Le sac est chaud, un peu gras.
+papa|Merci, Mila.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Ça sent le beurre et le four.
+enfant-f|Le croissant est à moi.
+maman|Il est dans tes mains.
+narrateur|Mila pose une main sur le sac.
+narrateur|Le papier est un peu rêche.
+narrateur|Sur le sac, un éclat de croissant tient.
+narrateur|La cloche se tait.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>papier</t>
+          <t>papier,cloche</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1805,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils restent sur le banc de pierre. Le soleil touche le papier. Tu veux un bout ? Oui, maman. S'il te plaît. Mila croque. C'est tiède. Ça sent la vanille. Merci, maman. Merci, Mila. Elle a des trous. Oui. Comme le fer. Une miette tombe près du banc. Pour le pigeon, peut-être. Il va revenir. Le fer souffle encore, plus loin. On garde le papier ? Il est encore chaud. Oui. Le pigeon revient près de la miette. Il l'a vue. Tout doux, maintenant.</t>
+          <t>Mila tire le sac trop vite. Je le montre, d'un coup ! Le papier glisse entre les doigts. Le croissant penche vers le sol. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila observe le pas, écoute la rue. Sur la pointe, un éclat de croissant luit. Là, près de la pointe. Mila tient le sac des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air tiède revient sur les joues. Mila serre le sac contre elle. Il reste chaud. On marche. Le sac penche, puis se cale. Je le tiens. On avance. Mila passe le pas. Le marbre reste derrière.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils restent sur le banc de pierre. Le soleil touche le papier. Tu veux un bout ? Oui, maman. S'il te plaît. Mila croque. C'est tiède. Ça sent la vanille. Merci, maman. Merci, Mila. Elle a des trous. Oui. Comme le fer. Une miette tombe près du banc. Pour le pigeon, peut-être. Il va revenir. Le fer souffle encore, plus loin. On garde le papier ? Il est encore chaud. Oui. Le pigeon revient près de la miette. Il l'a vue. Tout doux, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila tire le sac trop vite. Je le montre, d'un coup ! Le papier glisse entre les doigts. Le croissant penche vers le sol. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila observe le pas, écoute la rue. Sur la pointe, un &lt;emphasis level="moderate"&gt;éclat de croissant&lt;/emphasis&gt; luit. Là, près de la pointe. Mila tient le sac des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air tiède revient sur les joues. Mila serre le sac contre elle. Il reste chaud. On marche. Le sac penche, puis se cale. Je le tiens. On avance. Mila passe le pas. Le marbre reste derrière.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Fanny croque le croissant. Papa range le sac.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Mila tire le sac trop vite. Je le montre, d'un coup ! Le papier glisse entre les doigts. Le croissant penche vers le sol. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila observe le pas, écoute la rue. Sur la pointe, un &lt;emphasis&gt;éclat de croissant&lt;/emphasis&gt; luit. Là, près de la pointe. Mila tient le sac des deux mains. Le papier est rêche, un peu chaud. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On sort ? Oui, maman. La porte s'ouvre. La cloche fait ding. L'air tiède revient sur les joues. Mila serre le sac contre elle. Il reste chaud. On marche. Le sac penche, puis se cale. Je le tiens. On avance. Mila passe le pas. Le marbre reste derrière.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1827,30 +1862,34 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1859,28 +1898,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de croissant</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1889,51 +1932,62 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_croissant; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils restent sur le banc de pierre.
-narrateur|Le soleil touche le papier.
-maman|Tu veux un bout ?
+          <t>narrateur|Mila tire le sac trop vite.
+enfant-f|Je le montre, d'un coup !
+narrateur|Le papier glisse entre les doigts.
+narrateur|Le croissant penche vers le sol.
+enfant-f|Oh.
+narrateur|Mila avance les mains.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Mila observe le pas, écoute la rue.
+narrateur|Sur la pointe, un éclat de croissant luit.
+enfant-f|Là, près de la pointe.
+narrateur|Mila tient le sac des deux mains.
+narrateur|Le papier est rêche, un peu chaud.
+enfant-f|Il est chaud, papa.
+papa|Tu le portes jusqu'à la rue ?
+enfant-f|Oui, papa.
+maman|On sort ?
 enfant-f|Oui, maman.
-enfant-f|S'il te plaît.
-narrateur|Mila croque.
-narrateur|C'est tiède.
-narrateur|Ça sent la vanille.
-enfant-f|Merci, maman.
-papa|Merci, Mila.
-enfant-f|Elle a des trous.
-maman|Oui.
-maman|Comme le fer.
-narrateur|Une miette tombe près du banc.
-papa|Pour le pigeon, peut-être.
-enfant-f|Il va revenir.
-narrateur|Le fer souffle encore, plus loin.
-maman|On garde le papier ?
-enfant-f|Il est encore chaud.
-papa|Oui.
-narrateur|Le pigeon revient près de la miette.
-enfant-f|Il l'a vue.
-maman|Tout doux, maintenant.</t>
+narrateur|La porte s'ouvre.
+narrateur|La cloche fait ding.
+narrateur|L'air tiède revient sur les joues.
+narrateur|Mila serre le sac contre elle.
+enfant-f|Il reste chaud.
+papa|On marche.
+narrateur|Le sac penche, puis se cale.
+enfant-f|Je le tiens.
+maman|On avance.
+narrateur|Mila passe le pas.
+narrateur|Le marbre reste derrière.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>croque</t>
+          <t>pas,papier</t>
         </is>
       </c>
     </row>
@@ -1960,17 +2014,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le papier repose sur le banc. Il reste une miette, encore chaude. Bonne matinée, Mila. Elle était dorée, ta gaufre.</t>
+          <t>Le croissant brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur la pointe. Mila pose le sac contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Mila respire, plus large. On rentre ? Oui. Les joues de Mila se réchauffent. Le sac reste tiède sous la main. La farine tient sur la vitre. Elle ne tombe pas. Comme tout à l'heure ? Oui, maman. Le rayon est blanc, toi ? Oui, papa. Un éclat de croissant reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le papier repose sur le banc. Il reste une miette, encore chaude. Bonne matinée, Mila. Elle était dorée, ta gaufre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le croissant brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur la pointe. Mila pose le sac contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Mila respire, plus large. On rentre ? Oui. Les joues de Mila se réchauffent. Le sac reste tiède sous la main. La farine tient sur la vitre. Elle ne tombe pas. Comme tout à l'heure ? Oui, maman. Le rayon est blanc, toi ? Oui, papa. Un &lt;emphasis level="moderate"&gt;éclat de croissant&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le croissant brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur la pointe. Mila pose le sac contre le manteau. On le garde au chaud ? Oui, maman. Le four sentait bon. Il est contre toi. Une vapeur monte du papier. Mila respire, plus large. On rentre ? Oui. Les joues de Mila se réchauffent. Le sac reste tiède sous la main. La farine tient sur la vitre. Elle ne tombe pas. Comme tout à l'heure ? Oui, maman. Le rayon est blanc, toi ? Oui, papa. Un &lt;emphasis&gt;éclat de croissant&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2017,7 +2071,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2025,10 +2079,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2037,12 +2091,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2051,17 +2105,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de croissant</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2070,11 +2128,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2083,27 +2141,53 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_croissant_reste_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le papier repose sur le banc.
-narrateur|Il reste une miette, encore chaude.
-maman|Bonne matinée, Mila.
-papa|Elle était dorée, ta gaufre.</t>
+          <t>enfant-f|Le croissant brillait, papa.
+papa|Tu le vois, comme dans la boutique ?
+enfant-f|Oui, sur la pointe.
+narrateur|Mila pose le sac contre le manteau.
+maman|On le garde au chaud ?
+enfant-f|Oui, maman.
+enfant-f|Le four sentait bon.
+maman|Il est contre toi.
+narrateur|Une vapeur monte du papier.
+narrateur|Mila respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Mila se réchauffent.
+narrateur|Le sac reste tiède sous la main.
+narrateur|La farine tient sur la vitre.
+enfant-f|Elle ne tombe pas.
+maman|Comme tout à l'heure ?
+enfant-f|Oui, maman.
+papa|Le rayon est blanc, toi ?
+enfant-f|Oui, papa.
+narrateur|Un éclat de croissant reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pas</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2216,6 +2300,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>